<commit_message>
Ammo feedback and spawn evidence after the first Phase 2 playtest
The user's log verified boot, match start, the 10s intermission and a
17-creature wave 1 (DH-022, DH-024 done) but never reached "wave 1
cleared": they stopped after 22 seconds of shots not landing. Eighteen
confirmed hits plus misses against a 30-round magazine - the mag was
empty, the server dropped shots silently, and the client kept drawing
tracers. Nothing said press R.

- HitConfirm carries ammoLeft; new kinds "empty" (throttled to 1/s) and
  "reloaded"
- RifleClient auto-reloads on empty and prints ammo on every confirm
- WaveService prints "wave N fully spawned" with the cap-hold count so
  batched spawning has log evidence

Snapshot re-exported.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dino-Hunt-Tasks.xlsx
+++ b/Dino-Hunt-Tasks.xlsx
@@ -1869,13 +1869,13 @@
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J27" s="9" t="n"/>
       <c r="K27" s="8" t="inlineStr">
         <is>
-          <t>Config.Waves transcribes GDD §7 solo counts; species keys asserted against Config.Creatures at load.</t>
+          <t>User log 20:32:21: 'wave 1 started — 17 creatures across 1 lane(s)' = 12 Compsognathus + 5 Velociraptor. Composition verified.</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="I29" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J29" s="9" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="K29" s="8" t="inlineStr">
         <is>
-          <t>15s intermission (10s before wave 1). TimerEnd replicated via MatchState for the HUD countdown.</t>
+          <t>User log: 'intermission 10s before wave 1' at 20:32:11.6, wave started 20:32:21.6 — exactly 10s. HUD read phase Intermission. Same code path serves the 15s intermissions.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 2 playtest 2: waves 1-5 verified, dev commands, Pachy armour removed
The user's second log verifies the wave loop end to end: five waves
cleared in sequence with "cleared" firing on the last death every time,
scaling exact, and wave 2 throttled by the concurrency cap for 16 ticks
- the evidence DH-021 and DH-023 needed.

Findings acted on:
- 23 consecutive blocked shots on wave 3. The Pachycephalosaurus had a
  25-degree armour arc the GDD never gave it; its armour tutorial is the
  Triceratops at wave 7. Removed.
- Waves clear in 14-32s against a 40-65s target; noted for Phase 6
  balance, expected while creatures cannot attack.

Added DevCommands: Studio-only /wave N and /lose so victory and defeat
can be verified without a 25-minute run. WaveService's loop now drives
_nextWave so a jump can redirect it.

Snapshot re-exported. Tracker: DH-021, DH-023 done.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dino-Hunt-Tasks.xlsx
+++ b/Dino-Hunt-Tasks.xlsx
@@ -1816,7 +1816,7 @@
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>WaveService written: 20 finite waves, reservoir per wave, cleared when reservoir empty AND nothing alive. Awaiting user playtest logs.</t>
+          <t>User log 20:37-20:40: waves 1-5 cleared in 15/30/24/14/32s, each 'cleared' firing on the last death, intermission then next wave every time. Scaling exact (hp x1.07..x1.28). Wave-6 second lane load-checked, not played.</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J28" s="9" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="K28" s="8" t="inlineStr">
         <is>
-          <t>Reservoir drained 4 per 0.5s tick while CanSpawn(); cap never exceeded by construction.</t>
+          <t>User log: 'wave 2 fully spawned — 22 creatures in 12.7s, held by cap on 16 tick(s)'. Waves under the 18 cap held 0 ticks. Cap enforced by construction.</t>
         </is>
       </c>
     </row>

</xml_diff>